<commit_message>
added jira api and removed credentials
</commit_message>
<xml_diff>
--- a/LWS_reminder/plan.xlsx
+++ b/LWS_reminder/plan.xlsx
@@ -2,33 +2,49 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="167" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
@@ -42,12 +58,42 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -57,19 +103,29 @@
       <bottom style="thin"/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  <cellStyles count="2">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -432,33 +488,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>_parsed_date</t>
-        </is>
-      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="7" t="n">
         <v>45917</v>
       </c>
       <c r="B2" t="inlineStr">
@@ -471,188 +522,440 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="D2" s="3" t="n">
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="n">
         <v>45917</v>
       </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Enroll Postman Certification</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="n">
+        <v>45917</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Enroll postman qith AI cert</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="n">
+        <v>45917</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Engagement on Insta and linkedin</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="n">
+        <v>45918</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>post dropdown video</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="n">
+        <v>45918</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>complete postman expert cert</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="n">
+        <v>45918</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>complete postman with Ai Cert</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="n">
+        <v>45918</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Ready the content for auto suggest dropdowns HTML and Examples.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="n">
+        <v>45918</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Recod the video</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="n">
+        <v>45918</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Engagement on Insta and linkedin</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="n">
+        <v>46246</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">video on the reminder </t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="n">
+        <v>46246</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>call owner</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>12-08-2026</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>added a dummy task</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="n">
+        <v>46246</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>no status task</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>12-08-2026</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>added a task From UI</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>12-08-2026</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>dummy</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>12-08-2026</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>manual task added</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Created</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Due Date</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>SCRUM-6</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>this is a tast that is completed</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-08-12 16:37</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>45917</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SCRUM-5</t>
+        </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Enroll Postman Certification</t>
+          <t>task added in demo</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>45917</v>
-      </c>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-08-12 16:37</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>45917</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SCRUM-4</t>
+        </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Enroll postman qith AI cert</t>
+          <t>Subtask 2.1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>45917</v>
-      </c>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-08-12 13:02</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>45917</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SCRUM-3</t>
+        </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Engagement on Insta and linkedin</t>
+          <t>Task 3</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>45917</v>
-      </c>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-08-12 13:02</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>45918</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SCRUM-2</t>
+        </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>post dropdown video</t>
+          <t>Task 2</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="n">
-        <v>45918</v>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-08-12 13:02</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>45918</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SCRUM-1</t>
+        </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>complete postman expert cert</t>
+          <t>Task 1</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="n">
-        <v>45918</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>45918</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>complete postman with Ai Cert</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="n">
-        <v>45918</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>45918</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Ready the content for auto suggest dropdowns HTML and Examples.</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="n">
-        <v>45918</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="n">
-        <v>45918</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Recod the video</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="n">
-        <v>45918</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
-        <v>45918</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Engagement on Insta and linkedin</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="n">
-        <v>45918</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="n">
-        <v>46246</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">video on the reminder </t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="n">
-        <v>46246</v>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026-08-12 13:02</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>